<commit_message>
Perbaikan menu, opname, mutasi & export master data
- Menu index: filter kategori, urut by kategori+id, fix &amp; di label, fix penomoran
- Menu form: fix bahan tidak muncul saat edit (typo selected), fix qty desimal
- Menu show: kategori dari relasi, satuan di kolom tersendiri
- Menu destroy: handle recipe_group_id null (encoded 'kosong')
- Opname: urut bahan by kategori+id, system_qty filter by tanggal opname
- Opname model: missingPreviousOpname() — wajib approve opname bulan lalu
- MutationController: enforce cek opname bulan sebelumnya sebelum simpan
- master-exports: regenerate semua file Excel (bahan/kemasan/komposisi/menu/toko/supplier/user)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/master-exports/master_bahan_kemasan_komposisi.xlsx
+++ b/master-exports/master_bahan_kemasan_komposisi.xlsx
@@ -12,12 +12,12 @@
     <sheet name="Komposisi" sheetId="3" r:id="rId6"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1" forceFullCalc="1"/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="85">
   <si>
     <t>name</t>
   </si>
@@ -52,6 +52,15 @@
     <t>pcs</t>
   </si>
   <si>
+    <t>Tapioca Pearls</t>
+  </si>
+  <si>
+    <t>Nata De Coco</t>
+  </si>
+  <si>
+    <t>Natural Crystal Ball</t>
+  </si>
+  <si>
     <t>Non Dairy Creamer Sweet</t>
   </si>
   <si>
@@ -64,7 +73,22 @@
     <t>Pudding Powder</t>
   </si>
   <si>
-    <t>Tapioca Pearls</t>
+    <t>Black Tea (LOKAL)</t>
+  </si>
+  <si>
+    <t>Jasmine Tea (LOKAL)</t>
+  </si>
+  <si>
+    <t>Drinking Powder</t>
+  </si>
+  <si>
+    <t>Caramel Egg Flavor Solid Beverage</t>
+  </si>
+  <si>
+    <t>Strawberry Mixed Flavor Base Powder</t>
+  </si>
+  <si>
+    <t>Taro Flavored Solid Drink</t>
   </si>
   <si>
     <t>Fructose Syrup</t>
@@ -76,31 +100,13 @@
     <t>Sugar Syrup</t>
   </si>
   <si>
-    <t>Nata De Coco</t>
-  </si>
-  <si>
-    <t>Black Tea (LOKAL)</t>
-  </si>
-  <si>
-    <t>Jasmine Tea (LOKAL)</t>
-  </si>
-  <si>
-    <t>Drinking Powder</t>
-  </si>
-  <si>
     <t>Sugar Flavored Drink Puree</t>
   </si>
   <si>
-    <t>Natural Crystal Ball</t>
-  </si>
-  <si>
-    <t>Caramel Egg Flavor Solid Beverage</t>
-  </si>
-  <si>
-    <t>Strawberry Mixed Flavor Base Powder</t>
-  </si>
-  <si>
-    <t>Taro Flavored Solid Drink</t>
+    <t>Brown Sugar Syrup</t>
+  </si>
+  <si>
+    <t>Chocolate Syrup</t>
   </si>
   <si>
     <t>Mango Jam</t>
@@ -121,12 +127,6 @@
     <t>Peach Jam</t>
   </si>
   <si>
-    <t>Brown Sugar Syrup</t>
-  </si>
-  <si>
-    <t>Chocolate Syrup</t>
-  </si>
-  <si>
     <t>Cup 400</t>
   </si>
   <si>
@@ -239,6 +239,9 @@
   </si>
   <si>
     <t>Egg Pudding</t>
+  </si>
+  <si>
+    <t>Bubur Strawberry</t>
   </si>
   <si>
     <t>ingredient</t>
@@ -292,16 +295,34 @@
       <strike val="0"/>
       <u val="none"/>
       <sz val="11"/>
-      <color rgb="FF000000"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1e40af"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF065f46"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7c3aed"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -316,9 +337,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="3" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="4" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -618,8 +647,14 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:D61"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col min="1" max="1" width="42.418" bestFit="true" customWidth="true" style="0"/>
+    <col min="2" max="2" width="16.425" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="13.997" bestFit="true" customWidth="true" style="0"/>
+    <col min="4" max="4" width="13.997" bestFit="true" customWidth="true" style="0"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
@@ -685,7 +720,7 @@
         <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D5" t="s">
         <v>7</v>
@@ -693,13 +728,13 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D6" t="s">
         <v>7</v>
@@ -707,13 +742,13 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D7" t="s">
         <v>7</v>
@@ -721,13 +756,13 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s">
         <v>15</v>
-      </c>
-      <c r="B8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" t="s">
-        <v>6</v>
       </c>
       <c r="D8" t="s">
         <v>7</v>
@@ -741,7 +776,7 @@
         <v>5</v>
       </c>
       <c r="C9" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D9" t="s">
         <v>7</v>
@@ -749,13 +784,13 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
         <v>5</v>
       </c>
       <c r="C10" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D10" t="s">
         <v>7</v>
@@ -763,13 +798,13 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B11" t="s">
         <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="D11" t="s">
         <v>7</v>
@@ -777,13 +812,13 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B12" t="s">
         <v>5</v>
       </c>
       <c r="C12" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D12" t="s">
         <v>7</v>
@@ -791,13 +826,13 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B13" t="s">
         <v>5</v>
       </c>
       <c r="C13" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D13" t="s">
         <v>7</v>
@@ -805,13 +840,13 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B14" t="s">
         <v>5</v>
       </c>
       <c r="C14" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D14" t="s">
         <v>7</v>
@@ -819,13 +854,13 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B15" t="s">
         <v>5</v>
       </c>
       <c r="C15" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D15" t="s">
         <v>7</v>
@@ -833,13 +868,13 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B16" t="s">
         <v>5</v>
       </c>
       <c r="C16" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="D16" t="s">
         <v>7</v>
@@ -847,13 +882,13 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" t="s">
+        <v>5</v>
+      </c>
+      <c r="C17" t="s">
         <v>25</v>
-      </c>
-      <c r="B17" t="s">
-        <v>5</v>
-      </c>
-      <c r="C17" t="s">
-        <v>12</v>
       </c>
       <c r="D17" t="s">
         <v>7</v>
@@ -867,7 +902,7 @@
         <v>5</v>
       </c>
       <c r="C18" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="D18" t="s">
         <v>7</v>
@@ -881,7 +916,7 @@
         <v>5</v>
       </c>
       <c r="C19" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="D19" t="s">
         <v>7</v>
@@ -895,7 +930,7 @@
         <v>5</v>
       </c>
       <c r="C20" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D20" t="s">
         <v>7</v>
@@ -903,13 +938,13 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B21" t="s">
         <v>5</v>
       </c>
       <c r="C21" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D21" t="s">
         <v>7</v>
@@ -917,13 +952,13 @@
     </row>
     <row r="22" spans="1:4">
       <c r="A22" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" t="s">
+        <v>5</v>
+      </c>
+      <c r="C22" t="s">
         <v>31</v>
-      </c>
-      <c r="B22" t="s">
-        <v>5</v>
-      </c>
-      <c r="C22" t="s">
-        <v>29</v>
       </c>
       <c r="D22" t="s">
         <v>7</v>
@@ -937,7 +972,7 @@
         <v>5</v>
       </c>
       <c r="C23" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D23" t="s">
         <v>7</v>
@@ -951,7 +986,7 @@
         <v>5</v>
       </c>
       <c r="C24" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D24" t="s">
         <v>7</v>
@@ -965,7 +1000,7 @@
         <v>5</v>
       </c>
       <c r="C25" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="D25" t="s">
         <v>7</v>
@@ -979,7 +1014,7 @@
         <v>5</v>
       </c>
       <c r="C26" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="D26" t="s">
         <v>7</v>
@@ -1328,6 +1363,7 @@
       <c r="B51" t="s">
         <v>63</v>
       </c>
+      <c r="C51"/>
       <c r="D51" t="s">
         <v>7</v>
       </c>
@@ -1339,6 +1375,7 @@
       <c r="B52" t="s">
         <v>63</v>
       </c>
+      <c r="C52"/>
       <c r="D52" t="s">
         <v>7</v>
       </c>
@@ -1350,6 +1387,7 @@
       <c r="B53" t="s">
         <v>63</v>
       </c>
+      <c r="C53"/>
       <c r="D53" t="s">
         <v>7</v>
       </c>
@@ -1361,6 +1399,7 @@
       <c r="B54" t="s">
         <v>63</v>
       </c>
+      <c r="C54"/>
       <c r="D54" t="s">
         <v>7</v>
       </c>
@@ -1372,6 +1411,7 @@
       <c r="B55" t="s">
         <v>63</v>
       </c>
+      <c r="C55"/>
       <c r="D55" t="s">
         <v>7</v>
       </c>
@@ -1383,6 +1423,7 @@
       <c r="B56" t="s">
         <v>63</v>
       </c>
+      <c r="C56"/>
       <c r="D56" t="s">
         <v>7</v>
       </c>
@@ -1394,6 +1435,7 @@
       <c r="B57" t="s">
         <v>63</v>
       </c>
+      <c r="C57"/>
       <c r="D57" t="s">
         <v>7</v>
       </c>
@@ -1405,6 +1447,7 @@
       <c r="B58" t="s">
         <v>63</v>
       </c>
+      <c r="C58"/>
       <c r="D58" t="s">
         <v>7</v>
       </c>
@@ -1416,6 +1459,7 @@
       <c r="B59" t="s">
         <v>63</v>
       </c>
+      <c r="C59"/>
       <c r="D59" t="s">
         <v>7</v>
       </c>
@@ -1427,6 +1471,7 @@
       <c r="B60" t="s">
         <v>63</v>
       </c>
+      <c r="C60"/>
       <c r="D60" t="s">
         <v>7</v>
       </c>
@@ -1438,7 +1483,20 @@
       <c r="B61" t="s">
         <v>63</v>
       </c>
+      <c r="C61"/>
       <c r="D61" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4">
+      <c r="A62" t="s">
+        <v>74</v>
+      </c>
+      <c r="B62" t="s">
+        <v>63</v>
+      </c>
+      <c r="C62"/>
+      <c r="D62" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1465,22 +1523,29 @@
   </sheetPr>
   <dimension ref="A1:E50"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col min="1" max="1" width="42.418" bestFit="true" customWidth="true" style="0"/>
+    <col min="2" max="2" width="19.852" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="32.992" bestFit="true" customWidth="true" style="0"/>
+    <col min="4" max="4" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="5" max="5" width="17.567" bestFit="true" customWidth="true" style="0"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>78</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -1488,10 +1553,10 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D2">
         <v>1000</v>
@@ -1505,10 +1570,10 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D3">
         <v>8</v>
@@ -1522,10 +1587,10 @@
         <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D4">
         <v>16</v>
@@ -1536,13 +1601,13 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D5">
         <v>8</v>
@@ -1553,13 +1618,13 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D6">
         <v>10</v>
@@ -1570,13 +1635,13 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D7">
         <v>20</v>
@@ -1587,13 +1652,13 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C8" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D8">
         <v>16</v>
@@ -1604,13 +1669,13 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D9">
         <v>4</v>
@@ -1621,13 +1686,13 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="B10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C10" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D10">
         <v>4</v>
@@ -1638,13 +1703,13 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C11" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D11">
         <v>10</v>
@@ -1655,13 +1720,13 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B12" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C12" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D12">
         <v>120</v>
@@ -1672,13 +1737,13 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B13" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C13" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D13">
         <v>200</v>
@@ -1689,13 +1754,13 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B14" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C14" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D14">
         <v>15</v>
@@ -1706,13 +1771,13 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C15" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D15">
         <v>12</v>
@@ -1723,13 +1788,13 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C16" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D16">
         <v>20</v>
@@ -1740,13 +1805,13 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C17" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D17">
         <v>20</v>
@@ -1757,13 +1822,13 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B18" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D18">
         <v>30</v>
@@ -1774,13 +1839,13 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C19" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D19">
         <v>8</v>
@@ -1791,13 +1856,13 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C20" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D20">
         <v>20</v>
@@ -1808,13 +1873,13 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B21" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D21">
         <v>20</v>
@@ -1825,13 +1890,13 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B22" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C22" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D22">
         <v>20</v>
@@ -1842,13 +1907,13 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B23" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C23" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D23">
         <v>20</v>
@@ -1859,13 +1924,13 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B24" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C24" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D24">
         <v>20</v>
@@ -1876,13 +1941,13 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B25" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C25" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D25">
         <v>12</v>
@@ -1893,13 +1958,13 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B26" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C26" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D26">
         <v>12</v>
@@ -1913,10 +1978,10 @@
         <v>36</v>
       </c>
       <c r="B27" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C27" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D27">
         <v>20</v>
@@ -1930,10 +1995,10 @@
         <v>38</v>
       </c>
       <c r="B28" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C28" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D28">
         <v>20</v>
@@ -1947,10 +2012,10 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C29" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D29">
         <v>20</v>
@@ -1964,10 +2029,10 @@
         <v>40</v>
       </c>
       <c r="B30" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C30" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D30">
         <v>20</v>
@@ -1981,10 +2046,10 @@
         <v>41</v>
       </c>
       <c r="B31" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C31" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D31">
         <v>60</v>
@@ -1998,10 +2063,10 @@
         <v>42</v>
       </c>
       <c r="B32" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C32" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D32">
         <v>20</v>
@@ -2015,10 +2080,10 @@
         <v>43</v>
       </c>
       <c r="B33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C33" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D33">
         <v>20</v>
@@ -2032,10 +2097,10 @@
         <v>44</v>
       </c>
       <c r="B34" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C34" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D34">
         <v>10</v>
@@ -2049,10 +2114,10 @@
         <v>45</v>
       </c>
       <c r="B35" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C35" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D35">
         <v>80</v>
@@ -2066,10 +2131,10 @@
         <v>46</v>
       </c>
       <c r="B36" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C36" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D36">
         <v>60</v>
@@ -2083,10 +2148,10 @@
         <v>47</v>
       </c>
       <c r="B37" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C37" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D37">
         <v>25</v>
@@ -2100,10 +2165,10 @@
         <v>48</v>
       </c>
       <c r="B38" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C38" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D38">
         <v>6</v>
@@ -2117,10 +2182,10 @@
         <v>49</v>
       </c>
       <c r="B39" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C39" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D39">
         <v>50</v>
@@ -2134,10 +2199,10 @@
         <v>50</v>
       </c>
       <c r="B40" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C40" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D40">
         <v>500</v>
@@ -2151,10 +2216,10 @@
         <v>51</v>
       </c>
       <c r="B41" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C41" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D41">
         <v>500</v>
@@ -2168,10 +2233,10 @@
         <v>52</v>
       </c>
       <c r="B42" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C42" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D42">
         <v>30</v>
@@ -2185,10 +2250,10 @@
         <v>54</v>
       </c>
       <c r="B43" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C43" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D43">
         <v>24</v>
@@ -2202,10 +2267,10 @@
         <v>55</v>
       </c>
       <c r="B44" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C44" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D44">
         <v>20</v>
@@ -2219,10 +2284,10 @@
         <v>56</v>
       </c>
       <c r="B45" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C45" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D45">
         <v>20</v>
@@ -2236,10 +2301,10 @@
         <v>57</v>
       </c>
       <c r="B46" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C46" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D46">
         <v>40</v>
@@ -2253,10 +2318,10 @@
         <v>58</v>
       </c>
       <c r="B47" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C47" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D47">
         <v>40</v>
@@ -2270,10 +2335,10 @@
         <v>59</v>
       </c>
       <c r="B48" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C48" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D48">
         <v>40</v>
@@ -2287,10 +2352,10 @@
         <v>60</v>
       </c>
       <c r="B49" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C49" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D49">
         <v>40</v>
@@ -2304,10 +2369,10 @@
         <v>61</v>
       </c>
       <c r="B50" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C50" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D50">
         <v>40</v>
@@ -2337,18 +2402,23 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col min="1" max="1" width="28.136" bestFit="true" customWidth="true" style="0"/>
+    <col min="2" max="2" width="42.418" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="15.139" bestFit="true" customWidth="true" style="0"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>83</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -2356,7 +2426,7 @@
         <v>62</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C2">
         <v>0.27272727</v>
@@ -2367,7 +2437,7 @@
         <v>64</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C3">
         <v>0.3</v>
@@ -2378,7 +2448,7 @@
         <v>65</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C4">
         <v>0.47619048</v>
@@ -2389,7 +2459,7 @@
         <v>65</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="C5">
         <v>0.23809524</v>
@@ -2400,7 +2470,7 @@
         <v>66</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C6">
         <v>0.02553191</v>
@@ -2411,7 +2481,7 @@
         <v>67</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C7">
         <v>0.03703704</v>
@@ -2422,7 +2492,7 @@
         <v>68</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C8">
         <v>0.03508772</v>
@@ -2433,7 +2503,7 @@
         <v>68</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C9">
         <v>0.22807018</v>
@@ -2444,7 +2514,7 @@
         <v>69</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C10">
         <v>0.33333333</v>
@@ -2455,7 +2525,7 @@
         <v>70</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C11">
         <v>0.07692308</v>
@@ -2466,7 +2536,7 @@
         <v>71</v>
       </c>
       <c r="B12" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C12">
         <v>0.125</v>
@@ -2477,7 +2547,7 @@
         <v>71</v>
       </c>
       <c r="B13" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="C13">
         <v>0.125</v>
@@ -2488,7 +2558,7 @@
         <v>72</v>
       </c>
       <c r="B14" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C14">
         <v>0.09090909</v>
@@ -2499,7 +2569,7 @@
         <v>72</v>
       </c>
       <c r="B15" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C15">
         <v>0.09090909</v>
@@ -2510,7 +2580,7 @@
         <v>72</v>
       </c>
       <c r="B16" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="C16">
         <v>0.09090909</v>
@@ -2521,10 +2591,32 @@
         <v>73</v>
       </c>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C17">
         <v>0.14285714</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" t="s">
+        <v>74</v>
+      </c>
+      <c r="B18" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18">
+        <v>0.24778761</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" t="s">
+        <v>74</v>
+      </c>
+      <c r="B19" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19">
+        <v>0.04424779</v>
       </c>
     </row>
   </sheetData>

</xml_diff>